<commit_message>
updates at end of class
</commit_message>
<xml_diff>
--- a/assignment/data/lake_ice_off_data.xlsx
+++ b/assignment/data/lake_ice_off_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10309"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rqthomas/Documents/teaching/Environmental Data Science/github/lake-ice-template/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rqthomas/Documents/teaching/Environmental Data Science/github/lake-ice/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88A98B20-BDDD-6A49-B1E7-6144E0B2EC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B768DD97-42BC-FA40-8DC5-A189B9B77F37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51660" yWindow="500" windowWidth="22060" windowHeight="15160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="820" yWindow="760" windowWidth="33740" windowHeight="21580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="citation" sheetId="2" r:id="rId1"/>
@@ -33171,7 +33171,7 @@
         <v>15</v>
       </c>
       <c r="B2338">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C2338">
         <v>77</v>

</xml_diff>